<commit_message>
added regional reader for future project assignment of settings
</commit_message>
<xml_diff>
--- a/UploadTemplateTest.xlsx
+++ b/UploadTemplateTest.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hammertechcomau-my.sharepoint.com/personal/guy_accettura_hammertechglobal_com/Documents/Documents/PythonUploads/hammertech-worker-uploader/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="19" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB3F5EA5-F1E9-4859-8E6B-23ED8E54F9F5}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="8_{62830B75-0E58-4D82-B3B6-91C0511B9BE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{74DEB620-A5BC-48F9-AF57-56693FF90AFC}"/>
   <bookViews>
-    <workbookView xWindow="2115" yWindow="3000" windowWidth="21600" windowHeight="11175" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{016FCD56-390B-42A7-87FF-0F8E1F849A8B}"/>
   </bookViews>
   <sheets>
     <sheet name="Users" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="38">
   <si>
     <t>Email Address</t>
   </si>
@@ -140,9 +140,6 @@
     <t>Confidential Data</t>
   </si>
   <si>
-    <t>test@testing.com</t>
-  </si>
-  <si>
     <t>All perm</t>
   </si>
   <si>
@@ -155,10 +152,7 @@
     <t>All</t>
   </si>
   <si>
-    <t>testing@testing.com</t>
-  </si>
-  <si>
-    <t>(1) 7084081933</t>
+    <t>region@test.com</t>
   </si>
 </sst>
 </file>
@@ -541,7 +535,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9163D3E5-3974-4D02-94C9-F4EF4023A67A}">
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
@@ -593,69 +587,42 @@
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>34</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>35</v>
-      </c>
-      <c r="D2" t="s">
-        <v>36</v>
       </c>
       <c r="E2">
         <v>123</v>
       </c>
       <c r="F2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="H2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="I2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="J2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="K2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="B3" t="s">
-        <v>34</v>
-      </c>
-      <c r="C3" t="s">
-        <v>39</v>
-      </c>
-      <c r="D3" t="s">
         <v>36</v>
-      </c>
-      <c r="E3">
-        <v>456</v>
-      </c>
-      <c r="F3" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3" t="s">
-        <v>37</v>
-      </c>
-      <c r="J3" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="A2" r:id="rId1" xr:uid="{9DEDE0B0-2E97-4F55-B131-AF65B14899C4}"/>
-    <hyperlink ref="A3" r:id="rId2" xr:uid="{3B65D600-0F4B-42AB-95ED-D4B28E52CAF2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>